<commit_message>
[Feat] ItemData 테이블에 Id_Short 항목 추가
</commit_message>
<xml_diff>
--- a/Assets/Data/Table/Item/ItemData.xlsx
+++ b/Assets/Data/Table/Item/ItemData.xlsx
@@ -1,16 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28020"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5DB1C749-8AC7-492A-966B-4916AB43A602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KGA\source\repos\Project-FE\Assets\Data\Table\Item\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -31,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="109">
   <si>
     <t>Id</t>
   </si>
@@ -352,13 +356,32 @@
   </si>
   <si>
     <t>/Prefabs/BioFuel.prefab</t>
+  </si>
+  <si>
+    <t>Id_Short</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>hort</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -379,6 +402,26 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -394,7 +437,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -462,11 +505,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
@@ -478,6 +547,15 @@
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -813,58 +891,62 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I20"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J20"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="40.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.625" customWidth="1"/>
+    <col min="3" max="3" width="8.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>9</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>9</v>
@@ -873,541 +955,600 @@
         <v>9</v>
       </c>
       <c r="F2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>9</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:9">
+      <c r="J2" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="4">
-        <v>100</v>
-      </c>
       <c r="G3" s="4">
-        <v>0</v>
-      </c>
-      <c r="H3" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="J3" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5">
+        <v>2</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="4">
-        <v>100</v>
-      </c>
       <c r="G4" s="4">
-        <v>0</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>24</v>
+        <v>100</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:9">
+      <c r="J4" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5">
+        <v>3</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="4">
-        <v>100</v>
-      </c>
       <c r="G5" s="4">
-        <v>0</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>30</v>
+        <v>100</v>
+      </c>
+      <c r="H5" s="4">
+        <v>0</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="6" spans="1:9">
+      <c r="J5" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="4">
-        <v>100</v>
-      </c>
       <c r="G6" s="4">
-        <v>0</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>35</v>
+        <v>100</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="7" spans="1:9">
+      <c r="J6" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5">
+        <v>5</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="F7" s="4">
-        <v>100</v>
-      </c>
       <c r="G7" s="4">
-        <v>0</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>40</v>
+        <v>100</v>
+      </c>
+      <c r="H7" s="4">
+        <v>0</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="8" spans="1:9">
+      <c r="J7" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5">
+        <v>6</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="F8" s="4">
-        <v>100</v>
-      </c>
       <c r="G8" s="4">
-        <v>0</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>46</v>
+        <v>100</v>
+      </c>
+      <c r="H8" s="4">
+        <v>0</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="9" spans="1:9">
+      <c r="J8" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5">
+        <v>7</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="F9" s="4">
-        <v>100</v>
-      </c>
       <c r="G9" s="4">
-        <v>0</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>51</v>
+        <v>100</v>
+      </c>
+      <c r="H9" s="4">
+        <v>0</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="10" spans="1:9">
+      <c r="J9" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5">
+        <v>8</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="F10" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F10" s="4">
-        <v>100</v>
-      </c>
       <c r="G10" s="4">
-        <v>0</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>56</v>
+        <v>100</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0</v>
       </c>
       <c r="I10" s="4" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="11" spans="1:9">
+      <c r="J10" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="E11" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="F11" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="F11" s="4">
-        <v>100</v>
-      </c>
       <c r="G11" s="4">
-        <v>0</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>61</v>
+        <v>100</v>
+      </c>
+      <c r="H11" s="4">
+        <v>0</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="12" spans="1:9">
+      <c r="J11" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5">
+        <v>10</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="F12" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F12" s="4">
-        <v>100</v>
-      </c>
       <c r="G12" s="4">
-        <v>0</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>66</v>
+        <v>100</v>
+      </c>
+      <c r="H12" s="4">
+        <v>0</v>
       </c>
       <c r="I12" s="4" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="13" spans="1:9">
+      <c r="J12" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5">
+        <v>11</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="F13" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F13" s="4">
-        <v>100</v>
-      </c>
       <c r="G13" s="4">
-        <v>0</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>71</v>
+        <v>100</v>
+      </c>
+      <c r="H13" s="4">
+        <v>0</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="14" spans="1:9">
+      <c r="J13" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5">
+        <v>12</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="F14" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="F14" s="4">
-        <v>100</v>
-      </c>
       <c r="G14" s="4">
-        <v>0</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>76</v>
+        <v>100</v>
+      </c>
+      <c r="H14" s="4">
+        <v>0</v>
       </c>
       <c r="I14" s="4" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="15" spans="1:9">
+      <c r="J14" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5">
+        <v>13</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="D15" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="E15" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="F15" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F15" s="4">
-        <v>100</v>
-      </c>
       <c r="G15" s="4">
-        <v>0</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>81</v>
+        <v>100</v>
+      </c>
+      <c r="H15" s="4">
+        <v>0</v>
       </c>
       <c r="I15" s="4" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="16" spans="1:9">
+      <c r="J15" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5">
+        <v>14</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="D16" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="F16" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="F16" s="4">
-        <v>100</v>
-      </c>
       <c r="G16" s="4">
-        <v>0</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>86</v>
+        <v>100</v>
+      </c>
+      <c r="H16" s="4">
+        <v>0</v>
       </c>
       <c r="I16" s="4" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="17" spans="1:9">
+      <c r="J16" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5">
+        <v>15</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="E17" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="F17" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F17" s="4">
-        <v>100</v>
-      </c>
       <c r="G17" s="4">
-        <v>0</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>91</v>
+        <v>100</v>
+      </c>
+      <c r="H17" s="4">
+        <v>0</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="18" spans="1:9">
+      <c r="J17" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5">
+        <v>16</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="D18" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="E18" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="F18" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="F18" s="4">
-        <v>100</v>
-      </c>
       <c r="G18" s="4">
-        <v>0</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
+      </c>
+      <c r="H18" s="4">
+        <v>0</v>
       </c>
       <c r="I18" s="4" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="19" spans="1:9">
+      <c r="J18" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5">
+        <v>17</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="D19" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="E19" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="E19" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="F19" s="4">
+      <c r="F19" s="4" t="s">
         <v>100</v>
       </c>
       <c r="G19" s="4">
-        <v>0</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
+      </c>
+      <c r="H19" s="4">
+        <v>0</v>
       </c>
       <c r="I19" s="4" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="20" spans="1:9">
+      <c r="J19" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="5">
+        <v>18</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="D20" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="E20" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="F20" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="F20" s="4">
-        <v>100</v>
-      </c>
       <c r="G20" s="4">
+        <v>100</v>
+      </c>
+      <c r="H20" s="4">
         <v>1</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>106</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>106</v>
       </c>
+      <c r="J20" s="4" t="s">
+        <v>106</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>